<commit_message>
Update attendance spreadsheet ASS_CRN236396
Replace Administracion/Lista_Asistencia_ASS_CRN236396.xlsx with an updated binary Excel file containing revised attendance data for ASS_CRN236396. No textual diffs available since this is a binary spreadsheet update.
</commit_message>
<xml_diff>
--- a/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
+++ b/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\OneDrive\Documentos\GitHub\lc_arquitectura_de_sistemas_de_seguridad\Administracion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ddf5fb2bc65e958/Documentos/GitHub/lc_arquitectura_de_sistemas_de_seguridad/Administracion/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A38376A8-59C5-44D7-8BA9-AC04E8A4A2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -1403,9 +1403,6 @@
     <xf numFmtId="0" fontId="14" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1419,6 +1416,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1742,96 +1742,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-      <c r="M1" s="49"/>
-      <c r="N1" s="49"/>
-      <c r="O1" s="49"/>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="49"/>
-      <c r="R1" s="49"/>
-      <c r="S1" s="49"/>
-      <c r="T1" s="49"/>
-      <c r="U1" s="49"/>
-      <c r="V1" s="49"/>
-      <c r="W1" s="49"/>
-      <c r="X1" s="49"/>
-      <c r="Y1" s="49"/>
-      <c r="Z1" s="49"/>
-      <c r="AA1" s="49"/>
-      <c r="AB1" s="49"/>
-      <c r="AC1" s="49"/>
-      <c r="AD1" s="49"/>
-      <c r="AE1" s="49"/>
-      <c r="AF1" s="49"/>
-      <c r="AG1" s="49"/>
-      <c r="AH1" s="49"/>
-      <c r="AI1" s="49"/>
-      <c r="AJ1" s="49"/>
-      <c r="AK1" s="49"/>
-      <c r="AL1" s="49"/>
-      <c r="AM1" s="49"/>
-      <c r="AN1" s="49"/>
-      <c r="AO1" s="49"/>
-      <c r="AP1" s="49"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
+      <c r="U1" s="48"/>
+      <c r="V1" s="48"/>
+      <c r="W1" s="48"/>
+      <c r="X1" s="48"/>
+      <c r="Y1" s="48"/>
+      <c r="Z1" s="48"/>
+      <c r="AA1" s="48"/>
+      <c r="AB1" s="48"/>
+      <c r="AC1" s="48"/>
+      <c r="AD1" s="48"/>
+      <c r="AE1" s="48"/>
+      <c r="AF1" s="48"/>
+      <c r="AG1" s="48"/>
+      <c r="AH1" s="48"/>
+      <c r="AI1" s="48"/>
+      <c r="AJ1" s="48"/>
+      <c r="AK1" s="48"/>
+      <c r="AL1" s="48"/>
+      <c r="AM1" s="48"/>
+      <c r="AN1" s="48"/>
+      <c r="AO1" s="48"/>
+      <c r="AP1" s="48"/>
     </row>
     <row r="2" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
-      <c r="M2" s="50"/>
-      <c r="N2" s="50"/>
-      <c r="O2" s="50"/>
-      <c r="P2" s="50"/>
-      <c r="Q2" s="50"/>
-      <c r="R2" s="50"/>
-      <c r="S2" s="50"/>
-      <c r="T2" s="50"/>
-      <c r="U2" s="50"/>
-      <c r="V2" s="50"/>
-      <c r="W2" s="50"/>
-      <c r="X2" s="50"/>
-      <c r="Y2" s="50"/>
-      <c r="Z2" s="50"/>
-      <c r="AA2" s="50"/>
-      <c r="AB2" s="50"/>
-      <c r="AC2" s="50"/>
-      <c r="AD2" s="50"/>
-      <c r="AE2" s="50"/>
-      <c r="AF2" s="50"/>
-      <c r="AG2" s="50"/>
-      <c r="AH2" s="50"/>
-      <c r="AI2" s="50"/>
-      <c r="AJ2" s="50"/>
-      <c r="AK2" s="50"/>
-      <c r="AL2" s="50"/>
-      <c r="AM2" s="50"/>
-      <c r="AN2" s="50"/>
-      <c r="AO2" s="50"/>
-      <c r="AP2" s="50"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="49"/>
+      <c r="R2" s="49"/>
+      <c r="S2" s="49"/>
+      <c r="T2" s="49"/>
+      <c r="U2" s="49"/>
+      <c r="V2" s="49"/>
+      <c r="W2" s="49"/>
+      <c r="X2" s="49"/>
+      <c r="Y2" s="49"/>
+      <c r="Z2" s="49"/>
+      <c r="AA2" s="49"/>
+      <c r="AB2" s="49"/>
+      <c r="AC2" s="49"/>
+      <c r="AD2" s="49"/>
+      <c r="AE2" s="49"/>
+      <c r="AF2" s="49"/>
+      <c r="AG2" s="49"/>
+      <c r="AH2" s="49"/>
+      <c r="AI2" s="49"/>
+      <c r="AJ2" s="49"/>
+      <c r="AK2" s="49"/>
+      <c r="AL2" s="49"/>
+      <c r="AM2" s="49"/>
+      <c r="AN2" s="49"/>
+      <c r="AO2" s="49"/>
+      <c r="AP2" s="49"/>
     </row>
     <row r="3" spans="1:42" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -1855,70 +1855,70 @@
       <c r="G3" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="H3" s="45" t="s">
+      <c r="H3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="45"/>
-      <c r="J3" s="46" t="s">
+      <c r="I3" s="50"/>
+      <c r="J3" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="46"/>
-      <c r="L3" s="45" t="s">
+      <c r="K3" s="45"/>
+      <c r="L3" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="M3" s="45"/>
-      <c r="N3" s="46" t="s">
+      <c r="M3" s="50"/>
+      <c r="N3" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="O3" s="46"/>
-      <c r="P3" s="45" t="s">
+      <c r="O3" s="45"/>
+      <c r="P3" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="Q3" s="45"/>
-      <c r="R3" s="46" t="s">
+      <c r="Q3" s="50"/>
+      <c r="R3" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="S3" s="46"/>
-      <c r="T3" s="45" t="s">
+      <c r="S3" s="45"/>
+      <c r="T3" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="U3" s="45"/>
-      <c r="V3" s="46" t="s">
+      <c r="U3" s="50"/>
+      <c r="V3" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="W3" s="46"/>
-      <c r="X3" s="45" t="s">
+      <c r="W3" s="45"/>
+      <c r="X3" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="Y3" s="45"/>
-      <c r="Z3" s="46" t="s">
+      <c r="Y3" s="50"/>
+      <c r="Z3" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="AA3" s="46"/>
-      <c r="AB3" s="45" t="s">
+      <c r="AA3" s="45"/>
+      <c r="AB3" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="AC3" s="45"/>
-      <c r="AD3" s="46" t="s">
+      <c r="AC3" s="50"/>
+      <c r="AD3" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="AE3" s="46"/>
-      <c r="AF3" s="45" t="s">
+      <c r="AE3" s="45"/>
+      <c r="AF3" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="AG3" s="45"/>
-      <c r="AH3" s="46" t="s">
+      <c r="AG3" s="50"/>
+      <c r="AH3" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="AI3" s="46"/>
-      <c r="AJ3" s="45" t="s">
+      <c r="AI3" s="45"/>
+      <c r="AJ3" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="AK3" s="45"/>
-      <c r="AL3" s="46" t="s">
+      <c r="AK3" s="50"/>
+      <c r="AL3" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="AM3" s="46"/>
+      <c r="AM3" s="45"/>
       <c r="AN3" s="4" t="s">
         <v>22</v>
       </c>
@@ -5464,12 +5464,12 @@
       </c>
     </row>
     <row r="33" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="47" t="s">
+      <c r="A33" s="46" t="s">
         <v>140</v>
       </c>
-      <c r="B33" s="47"/>
-      <c r="C33" s="47"/>
-      <c r="D33" s="47"/>
+      <c r="B33" s="46"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="46"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
@@ -5606,50 +5606,50 @@
       <c r="AP33" s="5"/>
     </row>
     <row r="34" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="48" t="s">
+      <c r="A34" s="47" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="48"/>
-      <c r="C34" s="48"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="48"/>
-      <c r="H34" s="48"/>
-      <c r="I34" s="48"/>
-      <c r="J34" s="48"/>
-      <c r="K34" s="48"/>
-      <c r="L34" s="48"/>
-      <c r="M34" s="48"/>
-      <c r="N34" s="48"/>
-      <c r="O34" s="48"/>
-      <c r="P34" s="48"/>
-      <c r="Q34" s="48"/>
-      <c r="R34" s="48"/>
-      <c r="S34" s="48"/>
-      <c r="T34" s="48"/>
-      <c r="U34" s="48"/>
-      <c r="V34" s="48"/>
-      <c r="W34" s="48"/>
-      <c r="X34" s="48"/>
-      <c r="Y34" s="48"/>
-      <c r="Z34" s="48"/>
-      <c r="AA34" s="48"/>
-      <c r="AB34" s="48"/>
-      <c r="AC34" s="48"/>
-      <c r="AD34" s="48"/>
-      <c r="AE34" s="48"/>
-      <c r="AF34" s="48"/>
-      <c r="AG34" s="48"/>
-      <c r="AH34" s="48"/>
-      <c r="AI34" s="48"/>
-      <c r="AJ34" s="48"/>
-      <c r="AK34" s="48"/>
-      <c r="AL34" s="48"/>
-      <c r="AM34" s="48"/>
-      <c r="AN34" s="48"/>
-      <c r="AO34" s="48"/>
-      <c r="AP34" s="48"/>
+      <c r="B34" s="47"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="47"/>
+      <c r="J34" s="47"/>
+      <c r="K34" s="47"/>
+      <c r="L34" s="47"/>
+      <c r="M34" s="47"/>
+      <c r="N34" s="47"/>
+      <c r="O34" s="47"/>
+      <c r="P34" s="47"/>
+      <c r="Q34" s="47"/>
+      <c r="R34" s="47"/>
+      <c r="S34" s="47"/>
+      <c r="T34" s="47"/>
+      <c r="U34" s="47"/>
+      <c r="V34" s="47"/>
+      <c r="W34" s="47"/>
+      <c r="X34" s="47"/>
+      <c r="Y34" s="47"/>
+      <c r="Z34" s="47"/>
+      <c r="AA34" s="47"/>
+      <c r="AB34" s="47"/>
+      <c r="AC34" s="47"/>
+      <c r="AD34" s="47"/>
+      <c r="AE34" s="47"/>
+      <c r="AF34" s="47"/>
+      <c r="AG34" s="47"/>
+      <c r="AH34" s="47"/>
+      <c r="AI34" s="47"/>
+      <c r="AJ34" s="47"/>
+      <c r="AK34" s="47"/>
+      <c r="AL34" s="47"/>
+      <c r="AM34" s="47"/>
+      <c r="AN34" s="47"/>
+      <c r="AO34" s="47"/>
+      <c r="AP34" s="47"/>
     </row>
     <row r="35" spans="1:42" x14ac:dyDescent="0.25">
       <c r="AH35" s="26" t="s">
@@ -5658,6 +5658,10 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="AD3:AE3"/>
+    <mergeCell ref="AF3:AG3"/>
+    <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="AJ3:AK3"/>
     <mergeCell ref="AL3:AM3"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A34:AP34"/>
@@ -5674,10 +5678,6 @@
     <mergeCell ref="X3:Y3"/>
     <mergeCell ref="Z3:AA3"/>
     <mergeCell ref="AB3:AC3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="AF3:AG3"/>
-    <mergeCell ref="AH3:AI3"/>
-    <mergeCell ref="AJ3:AK3"/>
   </mergeCells>
   <conditionalFormatting sqref="AP6:AP32">
     <cfRule type="expression" dxfId="1" priority="2">
@@ -5707,16 +5707,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="48" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">

</xml_diff>